<commit_message>
change of a station's name
</commit_message>
<xml_diff>
--- a/Routes.xlsx
+++ b/Routes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eugk\Documents\iot\project\code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99469319-808E-4651-9AE7-A8DBE8DE98E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8470168-63BA-400C-BA0B-641C9511A80F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E451EE4A-2127-43C9-9A50-5536E739BF9B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="940" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="940" uniqueCount="190">
   <si>
     <t>Intracom</t>
   </si>
@@ -563,9 +563,6 @@
     <t>Haradros River</t>
   </si>
   <si>
-    <t>Polytechnic</t>
-  </si>
-  <si>
     <t>Conference Center</t>
   </si>
   <si>
@@ -594,6 +591,21 @@
   </si>
   <si>
     <t>University of Patras Chancellors Office</t>
+  </si>
+  <si>
+    <t>38.27920089206051, 21.76724285398675</t>
+  </si>
+  <si>
+    <t>38.281657955154586, 21.770596375604853</t>
+  </si>
+  <si>
+    <t>38.284356703219245, 21.77277117748854</t>
+  </si>
+  <si>
+    <t>38.28977270490379, 21.78496964937884</t>
+  </si>
+  <si>
+    <t>Polytechnio</t>
   </si>
 </sst>
 </file>
@@ -991,13 +1003,13 @@
   <sheetData>
     <row r="1" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.3">
@@ -2317,7 +2329,7 @@
         <v>139</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>42</v>
@@ -3098,7 +3110,7 @@
     </row>
     <row r="69" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B69" t="s">
-        <v>77</v>
+        <v>185</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>161</v>
@@ -3394,7 +3406,7 @@
     </row>
     <row r="79" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B79" s="1" t="s">
-        <v>77</v>
+        <v>186</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>163</v>
@@ -3513,7 +3525,7 @@
     </row>
     <row r="83" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B83" s="1" t="s">
-        <v>77</v>
+        <v>187</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>164</v>
@@ -4131,7 +4143,7 @@
         <v>114</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D104" t="s">
         <v>70</v>
@@ -4192,7 +4204,7 @@
         <v>116</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>175</v>
+        <v>189</v>
       </c>
       <c r="D106" t="s">
         <v>71</v>
@@ -4250,10 +4262,10 @@
     </row>
     <row r="108" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B108" t="s">
-        <v>77</v>
+        <v>188</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D108" t="s">
         <v>72</v>
@@ -4401,7 +4413,7 @@
         <v>122</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D113" t="s">
         <v>73</v>
@@ -4520,7 +4532,7 @@
         <v>126</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D117" t="s">
         <v>74</v>
@@ -4581,7 +4593,7 @@
         <v>128</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D119" t="s">
         <v>75</v>
@@ -4700,7 +4712,7 @@
         <v>132</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D123" t="s">
         <v>76</v>

</xml_diff>